<commit_message>
Candidatura FIFG 2027: presentazione opzionale e struttura nella risposta Host city
Presentazione di 12 slide 16:9 nella grafica delle brochure AIFG, con segnaposto
per i tracciati delle 18 buche e la mappa del percorso. Nel modulo Excel la voce
Host city descrive la posizione, i tre percorsi, lo Sheraton e la navetta.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EyPNUovAmh6SswiH9hVfN
</commit_message>
<xml_diff>
--- a/candidature/FIFG_2027_FIFG500_Italy_Bid_Response_Form.xlsx
+++ b/candidature/FIFG_2027_FIFG500_Italy_Bid_Response_Form.xlsx
@@ -299,10 +299,10 @@
     <t xml:space="preserve">Host city, region and country</t>
   </si>
   <si>
-    <t xml:space="preserve">Rome, Lazio, Italy – Golf Club Parco de' Medici</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Venue in the south-west of Rome (EUR / Magliana area), between Rome city centre and Fiumicino Airport.</t>
+    <t xml:space="preserve">Rome, Lazio, Italy – Golf Club Parco de' Medici. Venue in the south-west of Rome (EUR / Magliana area), between Rome city centre and Fiumicino Airport.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The golf complex has three golf courses (White, Blue and Red nines, 27 holes) and the Sheraton Rome Parco de' Medici hotel inside the venue: players stay on site with no daily transfers. The hotel runs a shuttle service to Fiumicino Airport (approx. 12 km), making air travel easy, and the area is well served by public transport to central Rome.</t>
   </si>
   <si>
     <t xml:space="preserve">Bid leader — name and role</t>
@@ -750,11 +750,12 @@
     <numFmt numFmtId="169" formatCode="0"/>
     <numFmt numFmtId="170" formatCode="\€#,##0.00;[RED]&quot;-€&quot;#,##0.00;;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -770,12 +771,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -927,7 +922,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -951,113 +946,112 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="10" fillId="7" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="7" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="7" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="7" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="6" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Normal" xfId="20"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -1341,407 +1335,407 @@
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="31"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="5" t="s">
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
+      <c r="A13" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="s">
+      <c r="A14" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+      <c r="A15" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
     </row>
     <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5" t="s">
+      <c r="E18" s="6"/>
+      <c r="F18" s="6" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="s">
+      <c r="A19" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="8" t="n">
+      <c r="B19" s="9" t="n">
         <f aca="false">COUNTIF('Bidder Details'!D5:D16,"Complete")+COUNTIF('Dates &amp; Event'!D5:D11,"Complete")+COUNTIF('Courses &amp; Operations'!D5:D14,"Complete")+COUNTIF('Fees &amp; Services'!D5:D12,"Complete")+COUNTIF('Media &amp; Funding'!D8:D16,"Complete")+COUNTIF('Compliance &amp; Variances'!E6:E13,"Complete")+COUNTIF('Bidder Details'!D5:D16,"Variance")+COUNTIF('Dates &amp; Event'!D5:D11,"Variance")+COUNTIF('Courses &amp; Operations'!D5:D14,"Variance")+COUNTIF('Fees &amp; Services'!D5:D12,"Variance")+COUNTIF('Media &amp; Funding'!D8:D16,"Variance")+COUNTIF('Compliance &amp; Variances'!E6:E13,"Variance")</f>
         <v>37</v>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="D19" s="10" t="n">
         <f aca="false">IF((B19+B20)=0,0,B19/(B19+B20))</f>
         <v>0.755102040816327</v>
       </c>
-      <c r="E19" s="9"/>
-      <c r="F19" s="10" t="s">
+      <c r="E19" s="10"/>
+      <c r="F19" s="11" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="8" t="n">
+      <c r="B20" s="9" t="n">
         <f aca="false">COUNTIF('Bidder Details'!D5:D16,"Missing")+COUNTIF('Dates &amp; Event'!D5:D11,"Missing")+COUNTIF('Courses &amp; Operations'!D5:D14,"Missing")+COUNTIF('Fees &amp; Services'!D5:D12,"Missing")+COUNTIF('Media &amp; Funding'!D8:D16,"Missing")+COUNTIF('Compliance &amp; Variances'!E6:E13,"Missing")</f>
         <v>12</v>
       </c>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="12" t="s">
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="13" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="8" t="n">
+      <c r="B21" s="9" t="n">
         <f aca="false">COUNTIF('Bidder Details'!D5:D16,"Variance")+COUNTIF('Dates &amp; Event'!D5:D11,"Variance")+COUNTIF('Courses &amp; Operations'!D5:D14,"Variance")+COUNTIF('Fees &amp; Services'!D5:D12,"Variance")+COUNTIF('Media &amp; Funding'!D8:D16,"Variance")+COUNTIF('Compliance &amp; Variances'!E6:E13,"Variance")</f>
         <v>0</v>
       </c>
-      <c r="D21" s="11"/>
-      <c r="E21" s="11"/>
-      <c r="F21" s="13" t="s">
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+      <c r="A22" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="11" t="str">
+      <c r="B22" s="12" t="str">
         <f aca="false">IF(B20&gt;0,"Outstanding items",IF(B21&gt;0,"Review variances","Ready for submission"))</f>
         <v>Outstanding items</v>
       </c>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="14" t="s">
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="15" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="F25" s="5" t="s">
+      <c r="F25" s="6" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="n">
+      <c r="A26" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E26" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="F26" s="7" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="n">
+      <c r="A27" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="F27" s="7" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="n">
+      <c r="A28" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E28" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="F28" s="7" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="n">
+      <c r="A29" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F29" s="7" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="n">
+      <c r="A30" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="F30" s="7" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="n">
+      <c r="A31" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="F31" s="7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="n">
+      <c r="A32" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="F32" s="7" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1797,229 +1791,229 @@
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="39"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="11" t="str">
+      <c r="C5" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="12" t="str">
         <f aca="false">IF(C5="No","Optional",IF(B5&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E5" s="10"/>
+      <c r="E5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="11" t="str">
+      <c r="C6" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="12" t="str">
         <f aca="false">IF(C6="No","Optional",IF(B6&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E6" s="10"/>
+      <c r="E6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" s="11" t="str">
+      <c r="C7" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" s="12" t="str">
         <f aca="false">IF(C7="No","Optional",IF(B7&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E7" s="10"/>
+      <c r="E7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>86</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D8" s="11" t="str">
+      <c r="C8" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8" s="12" t="str">
         <f aca="false">IF(C8="No","Optional",IF(B8&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="11" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="11" t="str">
+      <c r="C9" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="12" t="str">
         <f aca="false">IF(C9="No","Optional",IF(B9&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="11" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="B10" s="10"/>
-      <c r="C10" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="11" t="str">
+      <c r="B10" s="11"/>
+      <c r="C10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="12" t="str">
         <f aca="false">IF(C10="No","Optional",IF(B10&lt;&gt;"","Complete","Missing"))</f>
         <v>Missing</v>
       </c>
-      <c r="E10" s="10"/>
+      <c r="E10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="10"/>
-      <c r="C11" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D11" s="11" t="str">
+      <c r="B11" s="11"/>
+      <c r="C11" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D11" s="12" t="str">
         <f aca="false">IF(C11="No","Optional",IF(B11&lt;&gt;"","Complete","Missing"))</f>
         <v>Missing</v>
       </c>
-      <c r="E11" s="10"/>
+      <c r="E11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D12" s="11" t="str">
+      <c r="B12" s="17"/>
+      <c r="C12" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="12" t="str">
         <f aca="false">IF(C12="No","Optional",IF(B12&lt;&gt;"","Complete","Missing"))</f>
         <v>Missing</v>
       </c>
-      <c r="E12" s="10"/>
+      <c r="E12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="B13" s="16"/>
-      <c r="C13" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D13" s="11" t="str">
+      <c r="B13" s="17"/>
+      <c r="C13" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="12" t="str">
         <f aca="false">IF(C13="No","Optional",IF(B13&lt;&gt;"","Complete","Missing"))</f>
         <v>Missing</v>
       </c>
-      <c r="E13" s="10"/>
+      <c r="E13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="B14" s="16"/>
-      <c r="C14" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" s="11" t="str">
+      <c r="B14" s="17"/>
+      <c r="C14" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="12" t="str">
         <f aca="false">IF(C14="No","Optional",IF(B14&lt;&gt;"","Complete","Missing"))</f>
         <v>Missing</v>
       </c>
-      <c r="E14" s="10"/>
+      <c r="E14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="B15" s="16"/>
-      <c r="C15" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D15" s="11" t="str">
+      <c r="B15" s="17"/>
+      <c r="C15" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="12" t="str">
         <f aca="false">IF(C15="No","Optional",IF(B15&lt;&gt;"","Complete","Missing"))</f>
         <v>Missing</v>
       </c>
-      <c r="E15" s="10"/>
+      <c r="E15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D16" s="11" t="str">
+      <c r="B16" s="11"/>
+      <c r="C16" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="12" t="str">
         <f aca="false">IF(C16="No","Optional",IF(B16&lt;&gt;"","Complete","Missing"))</f>
         <v>Missing</v>
       </c>
-      <c r="E16" s="10"/>
+      <c r="E16" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2064,165 +2058,165 @@
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="39"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="11" t="str">
+      <c r="C5" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="12" t="str">
         <f aca="false">IF(C5="No","Optional",IF(B5&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="11" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="11" t="str">
+      <c r="C6" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="12" t="str">
         <f aca="false">IF(C6="No","Optional",IF(B6&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="11" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" s="11" t="str">
+      <c r="C7" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" s="12" t="str">
         <f aca="false">IF(C7="No","Optional",IF(B7&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="11" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <v>144</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D8" s="11" t="str">
+      <c r="C8" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8" s="12" t="str">
         <f aca="false">IF(C8="No","Optional",IF(B8&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="11" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="16" t="s">
         <v>111</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="11" t="str">
+      <c r="B9" s="11"/>
+      <c r="C9" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="12" t="str">
         <f aca="false">IF(C9="No","Optional",IF(B9&lt;&gt;"","Complete","Missing"))</f>
         <v>Missing</v>
       </c>
-      <c r="E9" s="10"/>
+      <c r="E9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="11" t="str">
+      <c r="B10" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="12" t="str">
         <f aca="false">IF(C10="No","Optional",IF(B10&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="11" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="B11" s="10"/>
-      <c r="C11" s="8" t="s">
+      <c r="B11" s="11"/>
+      <c r="C11" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="D11" s="11" t="str">
+      <c r="D11" s="12" t="str">
         <f aca="false">IF(C11="No","Optional",IF(B11&lt;&gt;"","Complete","Missing"))</f>
         <v>Optional</v>
       </c>
-      <c r="E11" s="10"/>
+      <c r="E11" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2271,219 +2265,219 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="39"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="11" t="str">
+      <c r="C5" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="12" t="str">
         <f aca="false">IF(C5="No","Optional",IF(B5&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="11" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="16" t="s">
         <v>120</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="11" t="str">
+      <c r="C6" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="12" t="str">
         <f aca="false">IF(C6="No","Optional",IF(B6&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="11" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>123</v>
       </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="8" t="str">
+      <c r="B7" s="11"/>
+      <c r="C7" s="9" t="str">
         <f aca="false">IF(OR('Bidder Details'!B7="FIFG Masters",'Bidder Details'!B7="FIFG Major 1000"),"Yes","No")</f>
         <v>No</v>
       </c>
-      <c r="D7" s="11" t="str">
+      <c r="D7" s="12" t="str">
         <f aca="false">IF(C7="No","Optional",IF(B7&lt;&gt;"","Complete","Missing"))</f>
         <v>Optional</v>
       </c>
-      <c r="E7" s="10"/>
+      <c r="E7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>124</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="8" t="str">
+      <c r="B8" s="11"/>
+      <c r="C8" s="9" t="str">
         <f aca="false">IF(OR('Bidder Details'!B7="FIFG Masters",'Bidder Details'!B7="FIFG Major 1000"),"Yes","No")</f>
         <v>No</v>
       </c>
-      <c r="D8" s="11" t="str">
+      <c r="D8" s="12" t="str">
         <f aca="false">IF(C8="No","Optional",IF(B8&lt;&gt;"","Complete","Missing"))</f>
         <v>Optional</v>
       </c>
-      <c r="E8" s="10"/>
+      <c r="E8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="11" t="str">
+      <c r="C9" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="12" t="str">
         <f aca="false">IF(C9="No","Optional",IF(B9&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="11" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="11" t="str">
+      <c r="B10" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="12" t="str">
         <f aca="false">IF(C10="No","Optional",IF(B10&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="11" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>130</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D11" s="11" t="str">
+      <c r="B11" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D11" s="12" t="str">
         <f aca="false">IF(C11="No","Optional",IF(B11&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="11" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="16" t="s">
         <v>132</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D12" s="11" t="str">
+      <c r="C12" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="12" t="str">
         <f aca="false">IF(C12="No","Optional",IF(B12&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="11" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D13" s="11" t="str">
+      <c r="C13" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="12" t="str">
         <f aca="false">IF(C13="No","Optional",IF(B13&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="11" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" s="11" t="str">
+      <c r="C14" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="12" t="str">
         <f aca="false">IF(C14="No","Optional",IF(B14&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="11" t="s">
         <v>140</v>
       </c>
     </row>
@@ -2524,189 +2518,189 @@
   <dimension ref="A1:E12"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="39"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="B5" s="19" t="n">
+      <c r="B5" s="20" t="n">
         <v>230</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D5" s="11" t="str">
+      <c r="C5" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" s="12" t="str">
         <f aca="false">IF(C5="No","Optional",IF(B5&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="11" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="11" t="str">
+      <c r="C6" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="12" t="str">
         <f aca="false">IF(C6="No","Optional",IF(B6&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="11" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="B7" s="19" t="n">
+      <c r="B7" s="20" t="n">
         <v>4000</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" s="11" t="str">
+      <c r="C7" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" s="12" t="str">
         <f aca="false">IF(C7="No","Optional",IF(B7&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="11" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D8" s="11" t="str">
+      <c r="B8" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8" s="12" t="str">
         <f aca="false">IF(C8="No","Optional",IF(B8&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="11" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="11" t="str">
+      <c r="C9" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="12" t="str">
         <f aca="false">IF(C9="No","Optional",IF(B9&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="11" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="11" t="str">
+      <c r="C10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="12" t="str">
         <f aca="false">IF(C10="No","Optional",IF(B10&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="11" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="D11" s="11" t="str">
+      <c r="D11" s="12" t="str">
         <f aca="false">IF(C11="No","Optional",IF(B11&lt;&gt;"","Complete","Missing"))</f>
         <v>Optional</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="11" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="16" t="s">
         <v>160</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="D12" s="11" t="str">
+      <c r="D12" s="12" t="str">
         <f aca="false">IF(C12="No","Optional",IF(B12&lt;&gt;"","Complete","Missing"))</f>
         <v>Optional</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="11" t="s">
         <v>162</v>
       </c>
     </row>
@@ -2753,223 +2747,223 @@
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="39"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="11" t="s">
         <v>167</v>
       </c>
-      <c r="C8" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D8" s="11" t="str">
+      <c r="C8" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8" s="12" t="str">
         <f aca="false">IF(C8="No","Optional",IF(B8&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="11" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="B9" s="19" t="n">
+      <c r="B9" s="20" t="n">
         <v>25000</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D9" s="11" t="str">
+      <c r="C9" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D9" s="12" t="str">
         <f aca="false">IF(C9="No","Optional",IF(B9&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="11" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="16" t="s">
         <v>171</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="11" t="s">
         <v>172</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="11" t="str">
+      <c r="C10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="12" t="str">
         <f aca="false">IF(C10="No","Optional",IF(B10&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="11" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="B11" s="19" t="n">
+      <c r="B11" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D11" s="11" t="str">
+      <c r="C11" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D11" s="12" t="str">
         <f aca="false">IF(C11="No","Optional",IF(B11&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="11" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="11" t="s">
         <v>177</v>
       </c>
-      <c r="C12" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D12" s="11" t="str">
+      <c r="C12" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="12" t="str">
         <f aca="false">IF(C12="No","Optional",IF(B12&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="11" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D13" s="11" t="str">
+      <c r="C13" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="12" t="str">
         <f aca="false">IF(C13="No","Optional",IF(B13&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="11" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="16" t="s">
         <v>182</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D14" s="11" t="str">
+      <c r="C14" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="12" t="str">
         <f aca="false">IF(C14="No","Optional",IF(B14&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="11" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>185</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="C15" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D15" s="11" t="str">
+      <c r="C15" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="12" t="str">
         <f aca="false">IF(C15="No","Optional",IF(B15&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" s="11" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="11" t="s">
         <v>189</v>
       </c>
-      <c r="C16" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="D16" s="11" t="str">
+      <c r="C16" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D16" s="12" t="str">
         <f aca="false">IF(C16="No","Optional",IF(B16&lt;&gt;"","Complete","Missing"))</f>
         <v>Complete</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="11" t="s">
         <v>190</v>
       </c>
     </row>
@@ -3017,201 +3011,201 @@
   <dimension ref="A1:F13"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="32"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E6" s="11" t="str">
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E6" s="12" t="str">
         <f aca="false">IF(D6="No","Not applicable",IF(B6="Yes","Complete",IF(B6="No","Variance","Missing")))</f>
         <v>Missing</v>
       </c>
-      <c r="F6" s="10"/>
+      <c r="F6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="7" t="s">
         <v>198</v>
       </c>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E7" s="11" t="str">
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E7" s="12" t="str">
         <f aca="false">IF(D7="No","Not applicable",IF(B7="Yes","Complete",IF(B7="No","Variance","Missing")))</f>
         <v>Missing</v>
       </c>
-      <c r="F7" s="10"/>
+      <c r="F7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="7" t="s">
         <v>199</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="B8" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="D8" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E8" s="11" t="str">
+      <c r="D8" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E8" s="12" t="str">
         <f aca="false">IF(D8="No","Not applicable",IF(B8="Yes","Complete",IF(B8="No","Variance","Missing")))</f>
         <v>Complete</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="11" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" s="11" t="str">
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E9" s="12" t="str">
         <f aca="false">IF(D9="No","Not applicable",IF(B9="Yes","Complete",IF(B9="No","Variance","Missing")))</f>
         <v>Missing</v>
       </c>
-      <c r="F9" s="10"/>
+      <c r="F9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C10" s="10" t="s">
+      <c r="B10" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C10" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E10" s="11" t="str">
+      <c r="D10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E10" s="12" t="str">
         <f aca="false">IF(D10="No","Not applicable",IF(B10="Yes","Complete",IF(B10="No","Variance","Missing")))</f>
         <v>Complete</v>
       </c>
-      <c r="F10" s="10"/>
+      <c r="F10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>205</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C11" s="10" t="s">
+      <c r="B11" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="D11" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E11" s="11" t="str">
+      <c r="D11" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E11" s="12" t="str">
         <f aca="false">IF(D11="No","Not applicable",IF(B11="Yes","Complete",IF(B11="No","Variance","Missing")))</f>
         <v>Complete</v>
       </c>
-      <c r="F11" s="10"/>
+      <c r="F11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="C12" s="10" t="s">
+      <c r="B12" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E12" s="11" t="str">
+      <c r="D12" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E12" s="12" t="str">
         <f aca="false">IF(D12="No","Not applicable",IF(B12="Yes","Complete",IF(B12="No","Variance","Missing")))</f>
         <v>Complete</v>
       </c>
-      <c r="F12" s="10"/>
+      <c r="F12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>209</v>
       </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E13" s="11" t="str">
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="E13" s="12" t="str">
         <f aca="false">IF(D13="No","Not applicable",IF(B13="Yes","Complete",IF(B13="No","Variance","Missing")))</f>
         <v>Missing</v>
       </c>
-      <c r="F13" s="10"/>
+      <c r="F13" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3257,352 +3251,352 @@
   <dimension ref="A1:C31"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="13.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>214</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="16" t="s">
         <v>215</v>
       </c>
-      <c r="B6" s="8" t="str">
+      <c r="B6" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B5="","",'Bidder Details'!B5)</f>
         <v>Italy</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="B7" s="8" t="str">
+      <c r="B7" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B6="","",'Bidder Details'!B6)</f>
         <v>Region 3 (Europe)</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="B8" s="8" t="str">
+      <c r="B8" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B7="","",'Bidder Details'!B7)</f>
         <v>FIFG 500</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="16" t="s">
         <v>217</v>
       </c>
-      <c r="B9" s="8" t="str">
+      <c r="B9" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B9="","",'Bidder Details'!B9)</f>
-        <v>Rome, Lazio, Italy – Golf Club Parco de' Medici</v>
-      </c>
-      <c r="C9" s="8" t="s">
+        <v>Rome, Lazio, Italy – Golf Club Parco de' Medici. Venue in the south-west of Rome (EUR / Magliana area), between Rome city centre and Fiumicino Airport.</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="16" t="s">
         <v>218</v>
       </c>
-      <c r="B10" s="20" t="str">
+      <c r="B10" s="21" t="str">
         <f aca="false">IF('Dates &amp; Event'!B5="","",'Dates &amp; Event'!B5)</f>
         <v>2 July 2027 (official practice day)</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="16" t="s">
         <v>219</v>
       </c>
-      <c r="B11" s="20" t="str">
+      <c r="B11" s="21" t="str">
         <f aca="false">IF('Dates &amp; Event'!B6="","",'Dates &amp; Event'!B6)</f>
         <v>4 July 2027</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="9" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="16" t="s">
         <v>220</v>
       </c>
-      <c r="B12" s="21" t="n">
+      <c r="B12" s="22" t="n">
         <f aca="false">IF('Dates &amp; Event'!B7="","",'Dates &amp; Event'!B7)</f>
         <v>2</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="9" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="9" t="n">
         <f aca="false">IF('Dates &amp; Event'!B8="","",'Dates &amp; Event'!B8)</f>
         <v>144</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="9" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="16" t="s">
         <v>221</v>
       </c>
-      <c r="B14" s="8" t="str">
+      <c r="B14" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B12="","",'Bidder Details'!B12)</f>
         <v/>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>222</v>
       </c>
-      <c r="B15" s="8" t="str">
+      <c r="B15" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B13="","",'Bidder Details'!B13)</f>
         <v/>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>223</v>
       </c>
-      <c r="B16" s="8" t="str">
+      <c r="B16" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B14="","",'Bidder Details'!B14)</f>
         <v/>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="s">
+      <c r="A17" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="B17" s="8" t="str">
+      <c r="B17" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B15="","",'Bidder Details'!B15)</f>
         <v/>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="16" t="s">
         <v>225</v>
       </c>
-      <c r="B18" s="22" t="n">
+      <c r="B18" s="23" t="n">
         <f aca="false">IF('Fees &amp; Services'!B5="","",'Fees &amp; Services'!B5)</f>
         <v>230</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="B19" s="8" t="str">
+      <c r="B19" s="9" t="str">
         <f aca="false">IF('Fees &amp; Services'!B6="","",'Fees &amp; Services'!B6)</f>
         <v>EUR 200 – early-bird valid 1–31 March 2027</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
+      <c r="A20" s="16" t="s">
         <v>227</v>
       </c>
-      <c r="B20" s="21" t="n">
+      <c r="B20" s="22" t="n">
         <f aca="false">IF('Fees &amp; Services'!B9="","",'Fees &amp; Services'!B9)</f>
         <v>2</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="16" t="s">
         <v>228</v>
       </c>
-      <c r="B21" s="8" t="str">
+      <c r="B21" s="9" t="str">
         <f aca="false">IF('Fees &amp; Services'!B8="","",'Fees &amp; Services'!B8)</f>
         <v>Yes</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="16" t="s">
         <v>148</v>
       </c>
-      <c r="B22" s="22" t="n">
+      <c r="B22" s="23" t="n">
         <f aca="false">IF('Fees &amp; Services'!B7="","",'Fees &amp; Services'!B7)</f>
         <v>4000</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="B23" s="8" t="str">
+      <c r="B23" s="9" t="str">
         <f aca="false">IF('Fees &amp; Services'!B11="","",'Fees &amp; Services'!B11)</f>
         <v>Sheraton Rome Parco de' Medici (on site, walking distance to the course) – event rate to be agreed</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="16" t="s">
         <v>229</v>
       </c>
-      <c r="B24" s="8" t="str">
+      <c r="B24" s="9" t="str">
         <f aca="false">IF('Fees &amp; Services'!B12="","",'Fees &amp; Services'!B12)</f>
         <v>Fiumicino (FCO): approx. 12 km, 15–20 min by car. Ciampino (CIA): approx. 20 km, 30 min. Rome Termini: approx. 25–30 min.</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="9" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="16" t="s">
         <v>230</v>
       </c>
-      <c r="B25" s="22" t="n">
+      <c r="B25" s="23" t="n">
         <f aca="false">IF('Media &amp; Funding'!B9="","",'Media &amp; Funding'!B9)</f>
         <v>25000</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="9" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="s">
+      <c r="A26" s="16" t="s">
         <v>231</v>
       </c>
-      <c r="B26" s="22" t="n">
+      <c r="B26" s="23" t="n">
         <f aca="false">IF('Media &amp; Funding'!B11="","",'Media &amp; Funding'!B11)</f>
         <v>0</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="9" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="s">
+      <c r="A27" s="16" t="s">
         <v>232</v>
       </c>
-      <c r="B27" s="8" t="str">
+      <c r="B27" s="9" t="str">
         <f aca="false">IF('Media &amp; Funding'!B12="","",'Media &amp; Funding'!B12)</f>
         <v>Applications planned to Regione Lazio (sport and tourism events), Roma Capitale (major events, sport and tourism) and ENIT – Italian National Tourism Agency.</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="9" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="16" t="s">
         <v>233</v>
       </c>
-      <c r="B28" s="8" t="str">
+      <c r="B28" s="9" t="str">
         <f aca="false">IF('Media &amp; Funding'!B13="","",'Media &amp; Funding'!B13)</f>
         <v>Local and national sponsors to be approached after the award; in-kind support from the venue/hotel partner. Amounts promoted only once guaranteed in writing.</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="9" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="8" t="n">
+      <c r="B29" s="9" t="n">
         <f aca="false">'Read Me &amp; Status'!B21</f>
         <v>0</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="9" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B30" s="9" t="n">
+      <c r="B30" s="10" t="n">
         <f aca="false">'Read Me &amp; Status'!D19</f>
         <v>0.755102040816327</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="9" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="s">
+      <c r="A31" s="16" t="s">
         <v>235</v>
       </c>
-      <c r="B31" s="11" t="str">
+      <c r="B31" s="12" t="str">
         <f aca="false">'Read Me &amp; Status'!B22</f>
         <v>Outstanding items</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="9" t="s">
         <v>234</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Candidatura FIFG 2027: good standing con il cambio di leadership AIFG
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014EyPNUovAmh6SswiH9hVfN
</commit_message>
<xml_diff>
--- a/candidature/FIFG_2027_FIFG500_Italy_Bid_Response_Form.xlsx
+++ b/candidature/FIFG_2027_FIFG500_Italy_Bid_Response_Form.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="238">
   <si>
     <t xml:space="preserve">FIFG 2027 Masters, Majors and 500 — Bid Response &amp; Comparison Workbook</t>
   </si>
@@ -621,6 +621,12 @@
   </si>
   <si>
     <t xml:space="preserve">Member Country is in good standing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Democratic change of leadership of the Associazione Italiana FootGolf (AIFG), the Italian FIFG Member; new leadership mandate 2027–2029.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The new leadership is rebuilding the Italian FootGolf movement. Response from players and clubs (ASD) has been very positive: the presentation event of the new leadership, on 14–15 November 2026 at Il Pelagone Hotel &amp; Golf Resort, Gavorrano (GR), is already sold out.</t>
   </si>
   <si>
     <t xml:space="preserve">No overdue FIFG debts at the submission deadline</t>
@@ -1516,11 +1522,11 @@
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">COUNTIF('Bidder Details'!D5:D16,"Complete")+COUNTIF('Dates &amp; Event'!D5:D11,"Complete")+COUNTIF('Courses &amp; Operations'!D5:D14,"Complete")+COUNTIF('Fees &amp; Services'!D5:D12,"Complete")+COUNTIF('Media &amp; Funding'!D8:D16,"Complete")+COUNTIF('Compliance &amp; Variances'!E6:E13,"Complete")+COUNTIF('Bidder Details'!D5:D16,"Variance")+COUNTIF('Dates &amp; Event'!D5:D11,"Variance")+COUNTIF('Courses &amp; Operations'!D5:D14,"Variance")+COUNTIF('Fees &amp; Services'!D5:D12,"Variance")+COUNTIF('Media &amp; Funding'!D8:D16,"Variance")+COUNTIF('Compliance &amp; Variances'!E6:E13,"Variance")</f>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D19" s="10" t="n">
         <f aca="false">IF((B19+B20)=0,0,B19/(B19+B20))</f>
-        <v>0.755102040816327</v>
+        <v>0.775510204081633</v>
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="11" t="s">
@@ -1533,7 +1539,7 @@
       </c>
       <c r="B20" s="9" t="n">
         <f aca="false">COUNTIF('Bidder Details'!D5:D16,"Missing")+COUNTIF('Dates &amp; Event'!D5:D11,"Missing")+COUNTIF('Courses &amp; Operations'!D5:D14,"Missing")+COUNTIF('Fees &amp; Services'!D5:D12,"Missing")+COUNTIF('Media &amp; Funding'!D8:D16,"Missing")+COUNTIF('Compliance &amp; Variances'!E6:E13,"Missing")</f>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D20" s="12"/>
       <c r="E20" s="12"/>
@@ -3073,20 +3079,26 @@
       <c r="A6" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
+      <c r="B6" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>198</v>
+      </c>
       <c r="D6" s="9" t="s">
         <v>81</v>
       </c>
       <c r="E6" s="12" t="str">
         <f aca="false">IF(D6="No","Not applicable",IF(B6="Yes","Complete",IF(B6="No","Variance","Missing")))</f>
-        <v>Missing</v>
-      </c>
-      <c r="F6" s="11"/>
+        <v>Complete</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -3101,13 +3113,13 @@
     </row>
     <row r="8" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>81</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>81</v>
@@ -3117,12 +3129,12 @@
         <v>Complete</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="11"/>
@@ -3137,13 +3149,13 @@
     </row>
     <row r="10" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>81</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>81</v>
@@ -3156,13 +3168,13 @@
     </row>
     <row r="11" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>81</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>81</v>
@@ -3175,13 +3187,13 @@
     </row>
     <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>81</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>81</v>
@@ -3194,7 +3206,7 @@
     </row>
     <row r="13" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
@@ -3258,21 +3270,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -3282,15 +3294,15 @@
         <v>24</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B6" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B5="","",'Bidder Details'!B5)</f>
@@ -3314,7 +3326,7 @@
     </row>
     <row r="8" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B8" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B7="","",'Bidder Details'!B7)</f>
@@ -3326,7 +3338,7 @@
     </row>
     <row r="9" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B9" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B9="","",'Bidder Details'!B9)</f>
@@ -3338,7 +3350,7 @@
     </row>
     <row r="10" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B10" s="21" t="str">
         <f aca="false">IF('Dates &amp; Event'!B5="","",'Dates &amp; Event'!B5)</f>
@@ -3350,7 +3362,7 @@
     </row>
     <row r="11" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B11" s="21" t="str">
         <f aca="false">IF('Dates &amp; Event'!B6="","",'Dates &amp; Event'!B6)</f>
@@ -3362,7 +3374,7 @@
     </row>
     <row r="12" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B12" s="22" t="n">
         <f aca="false">IF('Dates &amp; Event'!B7="","",'Dates &amp; Event'!B7)</f>
@@ -3386,7 +3398,7 @@
     </row>
     <row r="14" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B14" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B12="","",'Bidder Details'!B12)</f>
@@ -3398,7 +3410,7 @@
     </row>
     <row r="15" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B15" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B13="","",'Bidder Details'!B13)</f>
@@ -3410,7 +3422,7 @@
     </row>
     <row r="16" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B16" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B14="","",'Bidder Details'!B14)</f>
@@ -3422,7 +3434,7 @@
     </row>
     <row r="17" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B17" s="9" t="str">
         <f aca="false">IF('Bidder Details'!B15="","",'Bidder Details'!B15)</f>
@@ -3434,7 +3446,7 @@
     </row>
     <row r="18" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B18" s="23" t="n">
         <f aca="false">IF('Fees &amp; Services'!B5="","",'Fees &amp; Services'!B5)</f>
@@ -3446,7 +3458,7 @@
     </row>
     <row r="19" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B19" s="9" t="str">
         <f aca="false">IF('Fees &amp; Services'!B6="","",'Fees &amp; Services'!B6)</f>
@@ -3458,7 +3470,7 @@
     </row>
     <row r="20" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B20" s="22" t="n">
         <f aca="false">IF('Fees &amp; Services'!B9="","",'Fees &amp; Services'!B9)</f>
@@ -3470,7 +3482,7 @@
     </row>
     <row r="21" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B21" s="9" t="str">
         <f aca="false">IF('Fees &amp; Services'!B8="","",'Fees &amp; Services'!B8)</f>
@@ -3506,7 +3518,7 @@
     </row>
     <row r="24" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="16" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B24" s="9" t="str">
         <f aca="false">IF('Fees &amp; Services'!B12="","",'Fees &amp; Services'!B12)</f>
@@ -3518,7 +3530,7 @@
     </row>
     <row r="25" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B25" s="23" t="n">
         <f aca="false">IF('Media &amp; Funding'!B9="","",'Media &amp; Funding'!B9)</f>
@@ -3530,7 +3542,7 @@
     </row>
     <row r="26" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="16" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B26" s="23" t="n">
         <f aca="false">IF('Media &amp; Funding'!B11="","",'Media &amp; Funding'!B11)</f>
@@ -3542,7 +3554,7 @@
     </row>
     <row r="27" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="16" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B27" s="9" t="str">
         <f aca="false">IF('Media &amp; Funding'!B12="","",'Media &amp; Funding'!B12)</f>
@@ -3554,7 +3566,7 @@
     </row>
     <row r="28" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B28" s="9" t="str">
         <f aca="false">IF('Media &amp; Funding'!B13="","",'Media &amp; Funding'!B13)</f>
@@ -3573,7 +3585,7 @@
         <v>0</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3582,22 +3594,22 @@
       </c>
       <c r="B30" s="10" t="n">
         <f aca="false">'Read Me &amp; Status'!D19</f>
-        <v>0.755102040816327</v>
+        <v>0.775510204081633</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="16" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B31" s="12" t="str">
         <f aca="false">'Read Me &amp; Status'!B22</f>
         <v>Outstanding items</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>